<commit_message>
update universal -SO prompt
update universal -SO prompt
</commit_message>
<xml_diff>
--- a/DataGen_Automation_Kit/output/Shipment_From_SO_updated.xlsx
+++ b/DataGen_Automation_Kit/output/Shipment_From_SO_updated.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4470" yWindow="2550" windowWidth="21600" windowHeight="11775" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,8 +16,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN31"/>
+  <dimension ref="A1:AN34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -659,13 +659,13 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D2" t="n">
-        <v>2000374</v>
+        <v>2000446</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -674,12 +674,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Etsy VS</t>
+          <t>Golden State Apparel</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Etsy-VS</t>
+          <t>wh-Golden-SA</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -687,14 +687,9 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Etsy-VS ( Etsy )</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>10008-260308-000007</t>
+          <t>90015-260311-000019</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -709,21 +704,21 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>CAMILA-06-BLACK-8.5</t>
+          <t>AVIANA-06-BLACK-5.5</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>FUR SLIPPER</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>FUR SLIPPER</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -732,22 +727,22 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="U2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>43.85</v>
-      </c>
-      <c r="W2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" s="5" t="n">
+        <v>195</v>
+      </c>
+      <c r="W2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y2" s="4" t="n">
-        <v>43.85</v>
+        <v>195</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -764,14 +759,9 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>CAMILA-06</t>
+          <t>AVIANA-06</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
@@ -780,7 +770,7 @@
         </is>
       </c>
       <c r="AK2" t="n">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
@@ -789,19 +779,19 @@
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>1Z7SJNNA9SHKD1QZNE</t>
+          <t>1Z17SJNNA9SHKD1QZN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D3" t="n">
-        <v>2000384</v>
+        <v>2000437</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -810,12 +800,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Mirakl Kohls</t>
+          <t>AMZ eCom</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Mirakl-Kohls</t>
+          <t>AMZ-eCom</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -825,12 +815,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Mirakl-Kohls ( Kohl's (By Mirakl) )</t>
+          <t>AMZ-eCom ( Amazon )</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>10013-260308-000017</t>
+          <t>10001-260311-000010</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -845,12 +835,17 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>FB3601737-3219UNFORGV-30-STD</t>
+          <t>ADELINE-02-PINK-9</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Denim Stretch High-Waist Slit Hem Jeans</t>
+          <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
       <c r="Q3" t="n">
@@ -868,17 +863,17 @@
       <c r="U3" t="n">
         <v>2</v>
       </c>
-      <c r="V3" s="4" t="n">
-        <v>47.52</v>
-      </c>
-      <c r="W3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="4" t="n">
-        <v>47.52</v>
+      <c r="V3" s="5" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="W3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="5" t="n">
+        <v>96.7</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -895,54 +890,39 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>Standards &amp; Practices</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>BOTTOM</t>
-        </is>
-      </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>FB3601737</t>
+          <t>ADELINE-02</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>3219UNFORGV</t>
+          <t>PINK</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>30</v>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>Women</t>
-        </is>
+        <v>9</v>
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>WMSIZE1</t>
+          <t>WOMEN</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>1Z297MR8F50351F6TY</t>
+          <t>1ZE297MR8F50351F6T</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D4" t="n">
-        <v>2000385</v>
+        <v>2000441</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -951,12 +931,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Mirakl HudsonsB</t>
+          <t>AMZ eCom</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB</t>
+          <t>AMZ-eCom</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -966,12 +946,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB ( Hudson's Bay Marketplace (By Mirakl) )</t>
+          <t>AMZ-eCom ( Amazon )</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>10005-260308-000018</t>
+          <t>10001-260311-000014</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -986,16 +966,21 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>FB3601737-3219UNFORGV-30-STD</t>
+          <t>AVIANA-06-WHITE-8</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>FUR SLIPPER</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Denim Stretch High-Waist Slit Hem Jeans</t>
+          <t>FUR SLIPPER</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -1004,22 +989,22 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U4" t="n">
-        <v>4</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>79.72</v>
-      </c>
-      <c r="W4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="4" t="n">
-        <v>79.72</v>
+        <v>2</v>
+      </c>
+      <c r="V4" s="5" t="n">
+        <v>38.74</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="5" t="n">
+        <v>38.74</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1036,54 +1021,39 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>Standards &amp; Practices</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>BOTTOM</t>
-        </is>
-      </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>FB3601737</t>
+          <t>AVIANA-06</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>3219UNFORGV</t>
+          <t>WHITE</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>30</v>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>Women</t>
-        </is>
+        <v>8</v>
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>WMSIZE1</t>
+          <t>WOMEN</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>505336380898</t>
+          <t>050533638089897</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D5" t="n">
-        <v>2000373</v>
+        <v>2000438</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1092,12 +1062,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Shopify</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Shopify</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1107,12 +1077,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Shopify ( Shopify )</t>
+          <t>JCPenney ( JC Penney (By CommerceHub) )</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>20001-260308-000006</t>
+          <t>30007-260311-000011</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1127,21 +1097,16 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>AVIANA-06-BEIGE-6.5</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>FUR SLIPPER</t>
+          <t>F13031C-1742VNTGBJ-30-STD</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>Cayden Vintage Beujolias Corduroy Skinny Jeans</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -1150,22 +1115,22 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U5" t="n">
-        <v>1</v>
-      </c>
-      <c r="V5" s="4" t="n">
-        <v>61.05</v>
-      </c>
-      <c r="W5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="4" t="n">
-        <v>61.05</v>
+        <v>2</v>
+      </c>
+      <c r="V5" s="5" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="5" t="n">
+        <v>50.5</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1182,39 +1147,47 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Standards &amp; Practices</t>
+        </is>
+      </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>AVIANA-06</t>
+          <t>F13031C</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>BEIGE</t>
+          <t>1742VNTGBJ</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>6.5</v>
+        <v>30</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>4</v>
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>WMSIZE1</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>1Z3ZCDBYRMV8ZA4AJO</t>
+          <t>1ZZCDBYRMV8ZA4AJO5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D6" t="n">
-        <v>2000368</v>
+        <v>2000434</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1223,12 +1196,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Macys</t>
+          <t>Shopify</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Macys</t>
+          <t>Shopify</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1238,12 +1211,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Macys ( Macy's (By CommerceHub) )</t>
+          <t>Shopify ( Shopify )</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>30005-260308-000001</t>
+          <t>20001-260311-000007</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1258,17 +1231,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>AVIANA-06-BEIGE-9</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>FUR SLIPPER</t>
+          <t>F13031C-1742VNTGDM-28-STD</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>Cayden Vintage Beujolias Corduroy Skinny Jeans</t>
         </is>
       </c>
       <c r="Q6" t="n">
@@ -1286,17 +1254,17 @@
       <c r="U6" t="n">
         <v>1</v>
       </c>
-      <c r="V6" s="4" t="n">
-        <v>37.81</v>
-      </c>
-      <c r="W6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="4" t="n">
-        <v>37.81</v>
+      <c r="V6" s="5" t="n">
+        <v>30.43</v>
+      </c>
+      <c r="W6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="5" t="n">
+        <v>30.43</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1313,39 +1281,52 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Standards &amp; Practices</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>BOTTOM</t>
+        </is>
+      </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>AVIANA-06</t>
+          <t>F13031C</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>BEIGE</t>
+          <t>1742VNTGDM</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>9</v>
+        <v>28</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>4</v>
       </c>
       <c r="AM6" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>WMSIZE1</t>
         </is>
       </c>
       <c r="AN6" t="inlineStr">
         <is>
-          <t>1Z5LBMBHLSL5RFVGYN</t>
+          <t>1ZLBMBHLSL5RFVGYN1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D7" t="n">
-        <v>2000381</v>
+        <v>2000443</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1354,12 +1335,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AMZ eCom</t>
+          <t>Golden State Apparel</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>AMZ-eCom</t>
+          <t>wh-Golden-SA</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1367,14 +1348,9 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>AMZ-eCom ( Amazon )</t>
-        </is>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>10001-260308-000014</t>
+          <t>90015-260311-000016</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1389,21 +1365,21 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ADELINE-03-GOLD-5.5</t>
+          <t>ASTRID-01-NUDE-8.5</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>BUCKLE FRONT FLAT SANDALS</t>
+          <t>SLIP ON SNEAKER</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>BUCKLE FRONT FLAT SANDALS</t>
+          <t>SLIP ON SNEAKER</t>
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -1412,22 +1388,22 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>45.55</v>
-      </c>
-      <c r="W7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y7" s="4" t="n">
-        <v>45.55</v>
+        <v>83</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1446,21 +1422,21 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>BEAST</t>
+          <t>BF</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>ADELINE-03</t>
+          <t>ASTRID-01</t>
         </is>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>GOLD</t>
+          <t>NUDE</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>5.5</v>
+        <v>8.5</v>
       </c>
       <c r="AM7" t="inlineStr">
         <is>
@@ -1469,19 +1445,19 @@
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>333090466884016</t>
+          <t>330904668840</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D8" t="n">
-        <v>2000376</v>
+        <v>2000443</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1490,12 +1466,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AMZ eCom</t>
+          <t>Golden State Apparel</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AMZ-eCom</t>
+          <t>wh-Golden-SA</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1503,14 +1479,9 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>AMZ-eCom ( Amazon )</t>
-        </is>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>10001-260308-000009</t>
+          <t>90015-260311-000016</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1525,16 +1496,21 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>FA13501DM-1608BLAU2-31-32</t>
+          <t>ADELINE-02-WHITE-10</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Maya Basic Dark Handsand Wash Midrise Skinny Jeans</t>
+          <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1543,22 +1519,22 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="U8" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>54.99</v>
-      </c>
-      <c r="W8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y8" s="4" t="n">
-        <v>54.99</v>
+        <v>138</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1575,54 +1551,39 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>Poetic Justice</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>BOTTOM</t>
-        </is>
-      </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>FA13501DM</t>
+          <t>ADELINE-02</t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>1608BLAU2</t>
+          <t>WHITE</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>31</v>
-      </c>
-      <c r="AL8" t="inlineStr">
-        <is>
-          <t>Women</t>
-        </is>
+        <v>10</v>
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>WMSIZE1</t>
+          <t>WOMEN</t>
         </is>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>1ZPJGGKA9RTYLAZ6ZC</t>
+          <t>330904668840</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D9" t="n">
-        <v>2000380</v>
+        <v>2000442</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1631,12 +1592,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Etsy VS</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Etsy-VS</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1646,12 +1607,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Etsy-VS ( Etsy )</t>
+          <t>eBay ( eBay )</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>10008-260308-000013</t>
+          <t>10004-260311-000015</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1666,21 +1627,21 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>AVIANA-06-WHITE-5</t>
+          <t>CORA-01-FUCH-8</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1689,22 +1650,22 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U9" t="n">
-        <v>4</v>
-      </c>
-      <c r="V9" s="4" t="n">
-        <v>105.84</v>
-      </c>
-      <c r="W9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y9" s="4" t="n">
-        <v>105.84</v>
+        <v>3</v>
+      </c>
+      <c r="V9" s="5" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="5" t="n">
+        <v>78.51000000000001</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1723,16 +1684,16 @@
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>AVIANA-06</t>
+          <t>CORA-01</t>
         </is>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>WHITE</t>
+          <t>FUCH</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AM9" t="inlineStr">
         <is>
@@ -1741,33 +1702,33 @@
       </c>
       <c r="AN9" t="inlineStr">
         <is>
-          <t>570909686840216</t>
+          <t>1ZG0PJGGKA9RTYLAZ6</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D10" t="n">
-        <v>2000377</v>
+        <v>2000445</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Regular SKU</t>
+          <t>Prepack SKU</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>JCPenney</t>
+          <t>Walmart eComm</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>JCPenney</t>
+          <t>Walmart-eComm</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1777,12 +1738,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>JCPenney ( JC Penney (By CommerceHub) )</t>
+          <t>Walmart-eComm ( Walmart )</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>30007-260308-000010</t>
+          <t>10002-260311-000018</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1797,17 +1758,17 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>CORA-01-YLW-7.5</t>
+          <t>AUSTIN-06-BLUSH-A12</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>CROSS FRONT SANDAL</t>
+          <t>SNEAKER</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>CROSS FRONT SANDAL</t>
+          <t>SNEAKER</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -1825,17 +1786,17 @@
       <c r="U10" t="n">
         <v>1</v>
       </c>
-      <c r="V10" s="4" t="n">
-        <v>18.92</v>
-      </c>
-      <c r="W10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y10" s="4" t="n">
-        <v>18.92</v>
+      <c r="V10" s="5" t="n">
+        <v>29.04</v>
+      </c>
+      <c r="W10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="5" t="n">
+        <v>29.04</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1854,16 +1815,13 @@
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>CORA-01</t>
+          <t>AUSTIN-06</t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>YLW</t>
-        </is>
-      </c>
-      <c r="AK10" t="n">
-        <v>7.5</v>
+          <t>BLUSH</t>
+        </is>
       </c>
       <c r="AM10" t="inlineStr">
         <is>
@@ -1872,19 +1830,19 @@
       </c>
       <c r="AN10" t="inlineStr">
         <is>
-          <t>1ZHGFGWF1LP6IIE9C4</t>
+          <t>075709096868402</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D11" t="n">
-        <v>2000383</v>
+        <v>2000434</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1893,12 +1851,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Walmart eComm</t>
+          <t>Shopify</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Walmart-eComm</t>
+          <t>Shopify</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1908,12 +1866,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Walmart-eComm ( Walmart )</t>
+          <t>Shopify ( Shopify )</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>10002-260308-000016</t>
+          <t>20001-260311-000007</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1928,16 +1886,21 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>F13031C-1742VNTGST-24-STD</t>
+          <t>CORA-01-CAME-10</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Cayden Vintage Beujolias Corduroy Skinny Jeans</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1946,22 +1909,22 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U11" t="n">
-        <v>4</v>
-      </c>
-      <c r="V11" s="4" t="n">
-        <v>61.68</v>
-      </c>
-      <c r="W11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y11" s="4" t="n">
-        <v>61.68</v>
+        <v>2</v>
+      </c>
+      <c r="V11" s="5" t="n">
+        <v>33.48</v>
+      </c>
+      <c r="W11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="5" t="n">
+        <v>33.48</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1978,47 +1941,39 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>Standards &amp; Practices</t>
-        </is>
-      </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>F13031C</t>
+          <t>CORA-01</t>
         </is>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>1742VNTGST</t>
+          <t>CAME</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>24</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>WMSIZE1</t>
+          <t>WOMEN</t>
         </is>
       </c>
       <c r="AN11" t="inlineStr">
         <is>
-          <t>1ZX5VNNV134JTHRSWT</t>
+          <t>1ZLBMBHLSL5RFVGYN1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D12" t="n">
-        <v>2000375</v>
+        <v>2000430</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2047,7 +2002,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>10013-260308-000008</t>
+          <t>10013-260311-000003</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -2062,16 +2017,16 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>F13031C-1742VNTGDM-25-STD</t>
+          <t>FA13501DM-1608BLAU2-30-32</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Cayden Vintage Beujolias Corduroy Skinny Jeans</t>
+          <t>Maya Basic Dark Handsand Wash Midrise Skinny Jeans</t>
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R12" t="n">
         <v>0</v>
@@ -2080,22 +2035,22 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U12" t="n">
-        <v>2</v>
-      </c>
-      <c r="V12" s="4" t="n">
-        <v>105.26</v>
-      </c>
-      <c r="W12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="4" t="n">
-        <v>105.26</v>
+        <v>4</v>
+      </c>
+      <c r="V12" s="5" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="W12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="5" t="n">
+        <v>52.8</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -2114,7 +2069,7 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Standards &amp; Practices</t>
+          <t>Poetic Justice</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
@@ -2124,19 +2079,21 @@
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>F13031C</t>
+          <t>FA13501DM</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>1742VNTGDM</t>
+          <t>1608BLAU2</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>25</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>4</v>
+        <v>30</v>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
@@ -2145,19 +2102,19 @@
       </c>
       <c r="AN12" t="inlineStr">
         <is>
-          <t>1Z32GW1BK6ONT0H2ER</t>
+          <t>1ZG0HGFGWF1LP6IIE9</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D13" t="n">
-        <v>2000374</v>
+        <v>2000435</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2166,12 +2123,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Etsy VS</t>
+          <t>AMZ eCom</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Etsy-VS</t>
+          <t>AMZ-eCom</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2181,12 +2138,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Etsy-VS ( Etsy )</t>
+          <t>AMZ-eCom ( Amazon )</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>10008-260308-000007</t>
+          <t>10001-260311-000008</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2201,21 +2158,21 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>AVIANA-06-BLACK-5</t>
+          <t>CORA-01-TAUP-7</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -2224,22 +2181,22 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U13" t="n">
-        <v>1</v>
-      </c>
-      <c r="V13" s="4" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="W13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" s="4" t="n">
-        <v>18.2</v>
+        <v>4</v>
+      </c>
+      <c r="V13" s="5" t="n">
+        <v>57.32</v>
+      </c>
+      <c r="W13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="5" t="n">
+        <v>57.32</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2258,16 +2215,16 @@
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>AVIANA-06</t>
+          <t>CORA-01</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>TAUP</t>
         </is>
       </c>
       <c r="AK13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AM13" t="inlineStr">
         <is>
@@ -2276,33 +2233,33 @@
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>1Z7SJNNA9SHKD1QZNE</t>
+          <t>1ZC4X5VNNV134JTHRS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D14" t="n">
-        <v>2000386</v>
+        <v>2000435</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Prepack SKU</t>
+          <t>Regular SKU</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Macys</t>
+          <t>AMZ eCom</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Macys</t>
+          <t>AMZ-eCom</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2312,12 +2269,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Macys ( Macy's (By CommerceHub) )</t>
+          <t>AMZ-eCom ( Amazon )</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>30005-260308-000019</t>
+          <t>10001-260311-000008</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2332,17 +2289,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>CAMILA-06-BLACK-B12</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>173451-1183CITIZEN-19-34</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>Susan Stretch Denim Skinny Jeans Medium Blue 5 Poc</t>
         </is>
       </c>
       <c r="Q14" t="n">
@@ -2360,17 +2312,17 @@
       <c r="U14" t="n">
         <v>1</v>
       </c>
-      <c r="V14" s="4" t="n">
-        <v>46.07</v>
-      </c>
-      <c r="W14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="4" t="n">
-        <v>46.07</v>
+      <c r="V14" s="5" t="n">
+        <v>44.39</v>
+      </c>
+      <c r="W14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="5" t="n">
+        <v>44.39</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2389,39 +2341,48 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>CAMILA-06</t>
-        </is>
+          <t>Standards &amp; Practices</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>BOTTOM</t>
+        </is>
+      </c>
+      <c r="AI14" t="n">
+        <v>173451</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>BLACK</t>
-        </is>
+          <t>1183CITIZEN</t>
+        </is>
+      </c>
+      <c r="AK14" t="n">
+        <v>19</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>4</v>
       </c>
       <c r="AM14" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>JNSIZE</t>
         </is>
       </c>
       <c r="AN14" t="inlineStr">
         <is>
-          <t>1Z4XOMJNZG5QUN9UR9</t>
+          <t>1ZC4X5VNNV134JTHRS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D15" t="n">
-        <v>2000377</v>
+        <v>2000447</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2430,12 +2391,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>JCPenney</t>
+          <t>Etsy VS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>JCPenney</t>
+          <t>Etsy-VS</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2445,12 +2406,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>JCPenney ( JC Penney (By CommerceHub) )</t>
+          <t>Etsy-VS ( Etsy )</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>30007-260308-000010</t>
+          <t>10008-260311-000020</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2465,16 +2426,16 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>F13031C-1742VNTGDM-26-STD</t>
+          <t>34478006-BLACK-2X-STD</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Cayden Vintage Beujolias Corduroy Skinny Jeans</t>
+          <t>Supersoft longline mongolian cashmere cardigan</t>
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -2483,22 +2444,22 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U15" t="n">
-        <v>1</v>
-      </c>
-      <c r="V15" s="4" t="n">
-        <v>56.24</v>
-      </c>
-      <c r="W15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="4" t="n">
-        <v>56.24</v>
+        <v>2</v>
+      </c>
+      <c r="V15" s="5" t="n">
+        <v>45.88</v>
+      </c>
+      <c r="W15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="5" t="n">
+        <v>45.88</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2522,45 +2483,47 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>BOTTOM</t>
-        </is>
-      </c>
-      <c r="AI15" t="inlineStr">
-        <is>
-          <t>F13031C</t>
-        </is>
+          <t>SWEATERS</t>
+        </is>
+      </c>
+      <c r="AI15" t="n">
+        <v>34478006</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>1742VNTGDM</t>
-        </is>
-      </c>
-      <c r="AK15" t="n">
-        <v>26</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>4</v>
+          <t>BLACK</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>2X</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
       </c>
       <c r="AM15" t="inlineStr">
         <is>
-          <t>WMSIZE1</t>
+          <t>WPSIZE</t>
         </is>
       </c>
       <c r="AN15" t="inlineStr">
         <is>
-          <t>1ZHGFGWF1LP6IIE9C4</t>
+          <t>1ZWT32GW1BK6ONT0H2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D16" t="n">
-        <v>2000373</v>
+        <v>2000432</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2569,12 +2532,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Shopify</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Shopify</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2584,12 +2547,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Shopify ( Shopify )</t>
+          <t>eBay ( eBay )</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>20001-260308-000006</t>
+          <t>10004-260311-000005</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2604,17 +2567,17 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>CAMILA-06-TAUPE-8.5</t>
+          <t>ADELINE-02-CAMEL-9.5</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
       <c r="Q16" t="n">
@@ -2632,17 +2595,17 @@
       <c r="U16" t="n">
         <v>1</v>
       </c>
-      <c r="V16" s="4" t="n">
-        <v>34.99</v>
-      </c>
-      <c r="W16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y16" s="4" t="n">
-        <v>34.99</v>
+      <c r="V16" s="5" t="n">
+        <v>37.59</v>
+      </c>
+      <c r="W16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="5" t="n">
+        <v>37.59</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2659,23 +2622,18 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG16" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>CAMILA-06</t>
+          <t>ADELINE-02</t>
         </is>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>TAUPE</t>
+          <t>CAMEL</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="AM16" t="inlineStr">
         <is>
@@ -2684,19 +2642,19 @@
       </c>
       <c r="AN16" t="inlineStr">
         <is>
-          <t>1Z3ZCDBYRMV8ZA4AJO</t>
+          <t>1ZER4XOMJNZG5QUN9U</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D17" t="n">
-        <v>2000370</v>
+        <v>2000436</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2705,12 +2663,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Etsy VS</t>
+          <t>Golden State Apparel</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Etsy-VS</t>
+          <t>wh-Golden-SA</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2718,14 +2676,9 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Etsy-VS ( Etsy )</t>
-        </is>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>10008-260308-000003</t>
+          <t>90015-260311-000009</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2740,21 +2693,16 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>AVIANA-06-BLACK-10</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>FUR SLIPPER</t>
+          <t>F13031C-1742VNTGCO-32-STD</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>Cayden Vintage Beujolias Corduroy Skinny Jeans</t>
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
@@ -2763,22 +2711,22 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="U17" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>140.46</v>
-      </c>
-      <c r="W17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X17" s="5" t="n">
+        <v>408</v>
+      </c>
+      <c r="W17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y17" s="4" t="n">
-        <v>140.46</v>
+        <v>408</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2795,39 +2743,47 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>Standards &amp; Practices</t>
+        </is>
+      </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>AVIANA-06</t>
+          <t>F13031C</t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>1742VNTGCO</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>10</v>
+        <v>32</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>4</v>
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>WMSIZE1</t>
         </is>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>1ZAUPAO1ZTZ2OJJXS1</t>
+          <t>1ZR9AUPAO1ZTZ2OJJX</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D18" t="n">
-        <v>2000371</v>
+        <v>2000444</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2836,12 +2792,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Squarespace</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Squarespace</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2851,12 +2807,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Squarespace ( Squarespace )</t>
+          <t>JCPenney ( JC Penney (By CommerceHub) )</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>20006-260308-000004</t>
+          <t>30007-260311-000017</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2871,16 +2827,21 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>173451-1183CITIZEN-9-STD</t>
+          <t>AUSTIN-06-BLACK-9.5</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>SNEAKER</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Susan Stretch Denim Skinny Jeans Medium Blue 5 Poc</t>
+          <t>SNEAKER</t>
         </is>
       </c>
       <c r="Q18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
@@ -2889,22 +2850,22 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U18" t="n">
-        <v>2</v>
-      </c>
-      <c r="V18" s="4" t="n">
-        <v>90.76000000000001</v>
-      </c>
-      <c r="W18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y18" s="4" t="n">
-        <v>90.76000000000001</v>
+        <v>1</v>
+      </c>
+      <c r="V18" s="5" t="n">
+        <v>69.73999999999999</v>
+      </c>
+      <c r="W18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="5" t="n">
+        <v>69.73999999999999</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2921,64 +2882,53 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>Standards &amp; Practices</t>
-        </is>
-      </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>BOTTOM</t>
-        </is>
-      </c>
-      <c r="AI18" t="n">
-        <v>173451</v>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>AUSTIN-06</t>
+        </is>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>1183CITIZEN</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>9</v>
-      </c>
-      <c r="AL18" t="n">
-        <v>4</v>
+        <v>9.5</v>
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>JNSIZE</t>
+          <t>WOMEN</t>
         </is>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>125324665239</t>
+          <t>631253246652398</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D19" t="n">
-        <v>2000368</v>
+        <v>2000432</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Prepack SKU</t>
+          <t>Regular SKU</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Macys</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Macys</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2988,12 +2938,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Macys ( Macy's (By CommerceHub) )</t>
+          <t>eBay ( eBay )</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>30005-260308-000001</t>
+          <t>10004-260311-000005</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -3008,21 +2958,16 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>ASTRID-01-BLUSH-A12</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>SLIP ON SNEAKER</t>
+          <t>FA13512DM-1847DPOCN-26-30</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>SLIP ON SNEAKER</t>
+          <t>Angie Stud Bling Pocket Low Rise Skinny Jeans</t>
         </is>
       </c>
       <c r="Q19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -3031,22 +2976,22 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U19" t="n">
-        <v>1</v>
-      </c>
-      <c r="V19" s="4" t="n">
-        <v>38.12</v>
-      </c>
-      <c r="W19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y19" s="4" t="n">
-        <v>38.12</v>
+        <v>2</v>
+      </c>
+      <c r="V19" s="5" t="n">
+        <v>92.86</v>
+      </c>
+      <c r="W19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="5" t="n">
+        <v>92.86</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -3065,39 +3010,52 @@
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>BF</t>
+          <t>Poetic Justice</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>BOTTOM</t>
         </is>
       </c>
       <c r="AI19" t="inlineStr">
         <is>
-          <t>ASTRID-01</t>
+          <t>FA13512DM</t>
         </is>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>BLUSH</t>
+          <t>1847DPOCN</t>
+        </is>
+      </c>
+      <c r="AK19" t="n">
+        <v>26</v>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>Women</t>
         </is>
       </c>
       <c r="AM19" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>WMSIZE1</t>
         </is>
       </c>
       <c r="AN19" t="inlineStr">
         <is>
-          <t>1Z5LBMBHLSL5RFVGYN</t>
+          <t>1ZER4XOMJNZG5QUN9U</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D20" t="n">
-        <v>2000376</v>
+        <v>2000445</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3106,12 +3064,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AMZ eCom</t>
+          <t>Walmart eComm</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>AMZ-eCom</t>
+          <t>Walmart-eComm</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -3121,12 +3079,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>AMZ-eCom ( Amazon )</t>
+          <t>Walmart-eComm ( Walmart )</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>10001-260308-000009</t>
+          <t>10002-260311-000018</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -3141,21 +3099,21 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>CORA-01-BLK-12</t>
+          <t>ADELINE-03-BROWN-8</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>CROSS FRONT SANDAL</t>
+          <t>BUCKLE FRONT FLAT SANDALS</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>CROSS FRONT SANDAL</t>
+          <t>BUCKLE FRONT FLAT SANDALS</t>
         </is>
       </c>
       <c r="Q20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -3164,22 +3122,22 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U20" t="n">
-        <v>1</v>
-      </c>
-      <c r="V20" s="4" t="n">
-        <v>18.02</v>
-      </c>
-      <c r="W20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y20" s="4" t="n">
-        <v>18.02</v>
+        <v>4</v>
+      </c>
+      <c r="V20" s="5" t="n">
+        <v>75.44</v>
+      </c>
+      <c r="W20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="5" t="n">
+        <v>75.44</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -3196,18 +3154,23 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>BEAST</t>
+        </is>
+      </c>
       <c r="AI20" t="inlineStr">
         <is>
-          <t>CORA-01</t>
+          <t>ADELINE-03</t>
         </is>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>BLK</t>
+          <t>BROWN</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AM20" t="inlineStr">
         <is>
@@ -3216,19 +3179,19 @@
       </c>
       <c r="AN20" t="inlineStr">
         <is>
-          <t>1ZPJGGKA9RTYLAZ6ZC</t>
+          <t>075709096868402</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D21" t="n">
-        <v>2000387</v>
+        <v>2000443</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3237,12 +3200,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Squarespace</t>
+          <t>Golden State Apparel</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Squarespace</t>
+          <t>wh-Golden-SA</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -3250,14 +3213,9 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Squarespace ( Squarespace )</t>
-        </is>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>20006-260308-000020</t>
+          <t>90015-260311-000016</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -3272,16 +3230,21 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>F13031C-1742VNTGCO-26-STD</t>
+          <t>CORA-01-LEOP-12</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Cayden Vintage Beujolias Corduroy Skinny Jeans</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="Q21" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
@@ -3290,22 +3253,22 @@
         <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="U21" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>65.04000000000001</v>
-      </c>
-      <c r="W21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X21" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="W21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y21" s="4" t="n">
-        <v>65.04000000000001</v>
+        <v>172</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -3322,47 +3285,39 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG21" t="inlineStr">
-        <is>
-          <t>Standards &amp; Practices</t>
-        </is>
-      </c>
       <c r="AI21" t="inlineStr">
         <is>
-          <t>F13031C</t>
+          <t>CORA-01</t>
         </is>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>1742VNTGCO</t>
+          <t>LEOP</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>26</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="AM21" t="inlineStr">
         <is>
-          <t>WMSIZE1</t>
+          <t>WOMEN</t>
         </is>
       </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>214752329062832</t>
+          <t>330904668840</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D22" t="n">
-        <v>2000372</v>
+        <v>2000446</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3371,12 +3326,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>Golden State Apparel</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>wh-Golden-SA</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -3384,14 +3339,9 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Magento ( Magento 2.x )</t>
-        </is>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>20003-260308-000005</t>
+          <t>90015-260311-000019</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3406,21 +3356,21 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>ADELINE-02-CAMEL-12</t>
+          <t>CORA-01-TAUP-11</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>WOVEN SLIDE SANDAL</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>WOVEN SLIDE SANDAL</t>
+          <t>CROSS FRONT SANDAL</t>
         </is>
       </c>
       <c r="Q22" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -3429,22 +3379,22 @@
         <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="U22" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>97.68000000000001</v>
-      </c>
-      <c r="W22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X22" s="5" t="n">
+        <v>129</v>
+      </c>
+      <c r="W22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y22" s="4" t="n">
-        <v>97.68000000000001</v>
+        <v>129</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3463,16 +3413,16 @@
       </c>
       <c r="AI22" t="inlineStr">
         <is>
-          <t>ADELINE-02</t>
+          <t>CORA-01</t>
         </is>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>CAMEL</t>
+          <t>TAUP</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AM22" t="inlineStr">
         <is>
@@ -3481,19 +3431,19 @@
       </c>
       <c r="AN22" t="inlineStr">
         <is>
-          <t>442184087492141</t>
+          <t>1Z17SJNNA9SHKD1QZN</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D23" t="n">
-        <v>2000381</v>
+        <v>2000429</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3502,12 +3452,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>AMZ eCom</t>
+          <t>Macys</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>AMZ-eCom</t>
+          <t>Macys</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -3517,12 +3467,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>AMZ-eCom ( Amazon )</t>
+          <t>Macys ( Macy's (By CommerceHub) )</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>10001-260308-000014</t>
+          <t>30005-260311-000002</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3537,17 +3487,12 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>AVIANA-06-WHITE-12</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>FUR SLIPPER</t>
+          <t>FA13512DM-1847DPOCN-28-32</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>Angie Stud Bling Pocket Low Rise Skinny Jeans</t>
         </is>
       </c>
       <c r="Q23" t="n">
@@ -3565,17 +3510,17 @@
       <c r="U23" t="n">
         <v>1</v>
       </c>
-      <c r="V23" s="4" t="n">
-        <v>20.15</v>
-      </c>
-      <c r="W23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y23" s="4" t="n">
-        <v>20.15</v>
+      <c r="V23" s="5" t="n">
+        <v>35.15</v>
+      </c>
+      <c r="W23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="5" t="n">
+        <v>35.15</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3592,39 +3537,54 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>Poetic Justice</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>BOTTOM</t>
+        </is>
+      </c>
       <c r="AI23" t="inlineStr">
         <is>
-          <t>AVIANA-06</t>
+          <t>FA13512DM</t>
         </is>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>WHITE</t>
+          <t>1847DPOCN</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>12</v>
+        <v>28</v>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
       </c>
       <c r="AM23" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>WMSIZE1</t>
         </is>
       </c>
       <c r="AN23" t="inlineStr">
         <is>
-          <t>333090466884016</t>
+          <t>214752329062832</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D24" t="n">
-        <v>2000382</v>
+        <v>2000447</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3633,12 +3593,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Veeqo Amazon</t>
+          <t>Etsy VS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Veeqo-Amazon</t>
+          <t>Etsy-VS</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3648,12 +3608,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Veeqo-Amazon ( Amazon(By Veeqo) )</t>
+          <t>Etsy-VS ( Etsy )</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>10016-260308-000015</t>
+          <t>10008-260311-000020</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -3668,17 +3628,12 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>AUSTIN-06-WHITE-9.5</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>SNEAKER</t>
+          <t>FA13501DM-1464KINGSC-31-32</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>SNEAKER</t>
+          <t>Maya Basic Dark Handsand Wash Midrise Skinny Jeans</t>
         </is>
       </c>
       <c r="Q24" t="n">
@@ -3696,17 +3651,17 @@
       <c r="U24" t="n">
         <v>1</v>
       </c>
-      <c r="V24" s="4" t="n">
-        <v>56.94</v>
-      </c>
-      <c r="W24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" s="4" t="n">
-        <v>56.94</v>
+      <c r="V24" s="5" t="n">
+        <v>77.51000000000001</v>
+      </c>
+      <c r="W24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="5" t="n">
+        <v>77.51000000000001</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3723,39 +3678,54 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>Poetic Justice</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>BOTTOM</t>
+        </is>
+      </c>
       <c r="AI24" t="inlineStr">
         <is>
-          <t>AUSTIN-06</t>
+          <t>FA13501DM</t>
         </is>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>WHITE</t>
+          <t>1464KINGSC</t>
         </is>
       </c>
       <c r="AK24" t="n">
-        <v>9.5</v>
+        <v>31</v>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
       </c>
       <c r="AM24" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>WMSIZE1</t>
         </is>
       </c>
       <c r="AN24" t="inlineStr">
         <is>
-          <t>1ZFNOSBEKPMXFQGCLT</t>
+          <t>1ZWT32GW1BK6ONT0H2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D25" t="n">
-        <v>2000369</v>
+        <v>2000431</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3764,12 +3734,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Etsy LS</t>
+          <t>Harbor West Collective</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Etsy-LS</t>
+          <t>wh-Harbor-WC</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3777,14 +3747,9 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Etsy-LS ( Etsy )</t>
-        </is>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>10008-260308-000002</t>
+          <t>90016-260311-000004</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3799,21 +3764,21 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>AVIANA-06-BEIGE-12</t>
+          <t>ADELINE-03-BLACK-11</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>BUCKLE FRONT FLAT SANDALS</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>FUR SLIPPER</t>
+          <t>BUCKLE FRONT FLAT SANDALS</t>
         </is>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
@@ -3822,22 +3787,22 @@
         <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="U25" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="W25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X25" s="5" t="n">
+        <v>296</v>
+      </c>
+      <c r="W25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y25" s="4" t="n">
-        <v>42.4</v>
+        <v>296</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3854,18 +3819,23 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>BEAST</t>
+        </is>
+      </c>
       <c r="AI25" t="inlineStr">
         <is>
-          <t>AVIANA-06</t>
+          <t>ADELINE-03</t>
         </is>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>BEIGE</t>
+          <t>BLACK</t>
         </is>
       </c>
       <c r="AK25" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AM25" t="inlineStr">
         <is>
@@ -3874,19 +3844,19 @@
       </c>
       <c r="AN25" t="inlineStr">
         <is>
-          <t>685999299378921</t>
+          <t>442184087492141</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D26" t="n">
-        <v>2000379</v>
+        <v>2000428</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -3895,12 +3865,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Mirakl HudsonsB</t>
+          <t>Macys</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB</t>
+          <t>Macys</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3910,12 +3880,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB ( Hudson's Bay Marketplace (By Mirakl) )</t>
+          <t>Macys ( Macy's (By CommerceHub) )</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>10005-260308-000012</t>
+          <t>30005-260311-000001</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3930,17 +3900,17 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>CAMILA-06-NUDE-6.5</t>
+          <t>ADELINE-03-GOLD-6.5</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>BUCKLE FRONT FLAT SANDALS</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>BUCKLE FRONT FLAT SANDALS</t>
         </is>
       </c>
       <c r="Q26" t="n">
@@ -3958,17 +3928,17 @@
       <c r="U26" t="n">
         <v>3</v>
       </c>
-      <c r="V26" s="4" t="n">
-        <v>45.54</v>
-      </c>
-      <c r="W26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y26" s="4" t="n">
-        <v>45.54</v>
+      <c r="V26" s="5" t="n">
+        <v>89.94</v>
+      </c>
+      <c r="W26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" s="5" t="n">
+        <v>89.94</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3987,17 +3957,17 @@
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>BEAST</t>
         </is>
       </c>
       <c r="AI26" t="inlineStr">
         <is>
-          <t>CAMILA-06</t>
+          <t>ADELINE-03</t>
         </is>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>NUDE</t>
+          <t>GOLD</t>
         </is>
       </c>
       <c r="AK26" t="n">
@@ -4010,19 +3980,19 @@
       </c>
       <c r="AN26" t="inlineStr">
         <is>
-          <t>184582324550</t>
+          <t>1ZFNOSBEKPMXFQGCLT</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D27" t="n">
-        <v>2000378</v>
+        <v>2000439</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4031,12 +4001,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Mirakl HudsonsB</t>
+          <t>Etsy VS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB</t>
+          <t>Etsy-VS</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -4046,12 +4016,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB ( Hudson's Bay Marketplace (By Mirakl) )</t>
+          <t>Etsy-VS ( Etsy )</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>10005-260308-000011</t>
+          <t>10008-260311-000012</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -4066,21 +4036,16 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>CAMILA-06-TAUPE-11</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>FA13501DM-RINSEWSFT-29-30</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>COSS FRONT SLIP ON SLIDES</t>
+          <t>Maya Basic Dark Handsand Wash Midrise Skinny Jeans</t>
         </is>
       </c>
       <c r="Q27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -4089,22 +4054,22 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U27" t="n">
-        <v>4</v>
-      </c>
-      <c r="V27" s="4" t="n">
-        <v>125.2</v>
-      </c>
-      <c r="W27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y27" s="4" t="n">
-        <v>125.2</v>
+        <v>1</v>
+      </c>
+      <c r="V27" s="5" t="n">
+        <v>17.03</v>
+      </c>
+      <c r="W27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" s="5" t="n">
+        <v>17.03</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -4123,56 +4088,66 @@
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>Poetic Justice</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>BOTTOM</t>
         </is>
       </c>
       <c r="AI27" t="inlineStr">
         <is>
-          <t>CAMILA-06</t>
+          <t>FA13501DM</t>
         </is>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>TAUPE</t>
+          <t>RINSEWSFT</t>
         </is>
       </c>
       <c r="AK27" t="n">
-        <v>11</v>
+        <v>29</v>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
       </c>
       <c r="AM27" t="inlineStr">
         <is>
-          <t>WOMEN</t>
+          <t>WMSIZE1</t>
         </is>
       </c>
       <c r="AN27" t="inlineStr">
         <is>
-          <t>582947026906</t>
+          <t>685999299378921</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D28" t="n">
-        <v>2000379</v>
+        <v>2000438</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Prepack SKU</t>
+          <t>Regular SKU</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Mirakl HudsonsB</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4182,12 +4157,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Mirakl-HudsonsB ( Hudson's Bay Marketplace (By Mirakl) )</t>
+          <t>JCPenney ( JC Penney (By CommerceHub) )</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>10005-260308-000012</t>
+          <t>30007-260311-000011</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4202,17 +4177,17 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>AUSTIN-06-WHITE-B12</t>
+          <t>CAMILA-06-GREEN-12</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>SNEAKER</t>
+          <t>COSS FRONT SLIP ON SLIDES</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>SNEAKER</t>
+          <t>COSS FRONT SLIP ON SLIDES</t>
         </is>
       </c>
       <c r="Q28" t="n">
@@ -4230,17 +4205,17 @@
       <c r="U28" t="n">
         <v>1</v>
       </c>
-      <c r="V28" s="4" t="n">
-        <v>69.03</v>
-      </c>
-      <c r="W28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y28" s="4" t="n">
-        <v>69.03</v>
+      <c r="V28" s="5" t="n">
+        <v>25.18</v>
+      </c>
+      <c r="W28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="5" t="n">
+        <v>25.18</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -4257,15 +4232,23 @@
           <t>$</t>
         </is>
       </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
       <c r="AI28" t="inlineStr">
         <is>
-          <t>AUSTIN-06</t>
+          <t>CAMILA-06</t>
         </is>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
-          <t>WHITE</t>
-        </is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>12</v>
       </c>
       <c r="AM28" t="inlineStr">
         <is>
@@ -4274,19 +4257,19 @@
       </c>
       <c r="AN28" t="inlineStr">
         <is>
-          <t>184582324550</t>
+          <t>1ZZCDBYRMV8ZA4AJO5</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46089</v>
+        <v>46092</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D29" t="n">
-        <v>2000369</v>
+        <v>2000429</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4295,12 +4278,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Etsy LS</t>
+          <t>Macys</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Etsy-LS</t>
+          <t>Macys</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -4310,12 +4293,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Etsy-LS ( Etsy )</t>
+          <t>Macys ( Macy's (By CommerceHub) )</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>10008-260308-000002</t>
+          <t>30005-260311-000002</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4330,16 +4313,21 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>173451-1183CITIZEN-5-STD</t>
+          <t>AVIANA-06-WHITE-12</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>FUR SLIPPER</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Susan Stretch Denim Skinny Jeans Medium Blue 5 Poc</t>
+          <t>FUR SLIPPER</t>
         </is>
       </c>
       <c r="Q29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
@@ -4348,22 +4336,22 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U29" t="n">
-        <v>1</v>
-      </c>
-      <c r="V29" s="4" t="n">
-        <v>32.28</v>
-      </c>
-      <c r="W29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y29" s="4" t="n">
-        <v>32.28</v>
+        <v>3</v>
+      </c>
+      <c r="V29" s="5" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="W29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="5" t="n">
+        <v>41.1</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
@@ -4380,50 +4368,39 @@
           <t>$</t>
         </is>
       </c>
-      <c r="AG29" t="inlineStr">
-        <is>
-          <t>Standards &amp; Practices</t>
-        </is>
-      </c>
-      <c r="AH29" t="inlineStr">
-        <is>
-          <t>BOTTOM</t>
-        </is>
-      </c>
-      <c r="AI29" t="n">
-        <v>173451</v>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>AVIANA-06</t>
+        </is>
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
-          <t>1183CITIZEN</t>
+          <t>WHITE</t>
         </is>
       </c>
       <c r="AK29" t="n">
-        <v>5</v>
-      </c>
-      <c r="AL29" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="AM29" t="inlineStr">
         <is>
-          <t>JNSIZE</t>
+          <t>WOMEN</t>
         </is>
       </c>
       <c r="AN29" t="inlineStr">
         <is>
-          <t>685999299378921</t>
+          <t>214752329062832</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46086</v>
+        <v>46092</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D30" t="n">
-        <v>2000318</v>
+        <v>2000441</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -4452,7 +4429,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>10001-260305-000011</t>
+          <t>10001-260311-000014</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4467,7 +4444,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>AVIANA-06-BLACK-8.5</t>
+          <t>AVIANA-06-WHITE-9</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -4481,7 +4458,7 @@
         </is>
       </c>
       <c r="Q30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -4490,22 +4467,22 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V30" s="5" t="n">
-        <v>65</v>
-      </c>
-      <c r="W30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X30" s="5" t="n">
+        <v>29.52</v>
+      </c>
+      <c r="W30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Y30" s="5" t="n">
-        <v>65</v>
+        <v>29.52</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4529,11 +4506,11 @@
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
-          <t>BLACK</t>
+          <t>WHITE</t>
         </is>
       </c>
       <c r="AK30" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="AM30" t="inlineStr">
         <is>
@@ -4542,19 +4519,19 @@
       </c>
       <c r="AN30" t="inlineStr">
         <is>
-          <t>712360626311804</t>
+          <t>050533638089897</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46086</v>
+        <v>46092</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>46091</v>
+        <v>46094</v>
       </c>
       <c r="D31" t="n">
-        <v>2000318</v>
+        <v>2000438</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -4563,12 +4540,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AMZ eCom</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>AMZ-eCom</t>
+          <t>JCPenney</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -4578,12 +4555,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>AMZ-eCom ( Amazon )</t>
+          <t>JCPenney ( JC Penney (By CommerceHub) )</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>10001-260305-000011</t>
+          <t>30007-260311-000011</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4598,82 +4575,477 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>ADELINE-02-WHITE-8</t>
+          <t>CORA-01-CAME-6</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
+          <t>CROSS FRONT SANDAL</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>CROSS FRONT SANDAL</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>2</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>2</v>
+      </c>
+      <c r="U31" t="n">
+        <v>2</v>
+      </c>
+      <c r="V31" s="5" t="n">
+        <v>29.42</v>
+      </c>
+      <c r="W31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="5" t="n">
+        <v>29.42</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>CORA-01</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>CAME</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>6</v>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>1ZZCDBYRMV8ZA4AJO5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2000439</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Regular SKU</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Etsy VS</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Etsy-VS</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Etsy-VS ( Etsy )</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>10008-260311-000012</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>CAMILA-06-NUDE-10</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>COSS FRONT SLIP ON SLIDES</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>COSS FRONT SLIP ON SLIDES</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>2</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>2</v>
+      </c>
+      <c r="U32" t="n">
+        <v>2</v>
+      </c>
+      <c r="V32" s="5" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="W32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="5" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>CAMILA-06</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>NUDE</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>10</v>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>685999299378921</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2000433</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Regular SKU</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Veeqo Amazon</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Veeqo-Amazon</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Veeqo-Amazon ( Amazon(By Veeqo) )</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>10016-260311-000006</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>ADELINE-02-CAMEL-5.5</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
           <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>WOVEN SLIDE SANDAL</t>
         </is>
       </c>
-      <c r="Q31" t="n">
+      <c r="Q33" t="n">
         <v>3</v>
       </c>
-      <c r="R31" t="n">
-        <v>0</v>
-      </c>
-      <c r="S31" t="n">
-        <v>0</v>
-      </c>
-      <c r="T31" t="n">
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
         <v>3</v>
       </c>
-      <c r="U31" t="n">
+      <c r="U33" t="n">
         <v>3</v>
       </c>
-      <c r="V31" s="4" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="W31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X31" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y31" s="4" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="Z31" t="inlineStr">
-        <is>
-          <t>$</t>
-        </is>
-      </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>$</t>
-        </is>
-      </c>
-      <c r="AB31" t="inlineStr">
-        <is>
-          <t>$</t>
-        </is>
-      </c>
-      <c r="AI31" t="inlineStr">
+      <c r="V33" s="5" t="n">
+        <v>123.03</v>
+      </c>
+      <c r="W33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" s="5" t="n">
+        <v>123.03</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AI33" t="inlineStr">
         <is>
           <t>ADELINE-02</t>
         </is>
       </c>
-      <c r="AJ31" t="inlineStr">
-        <is>
-          <t>WHITE</t>
-        </is>
-      </c>
-      <c r="AK31" t="n">
-        <v>8</v>
-      </c>
-      <c r="AM31" t="inlineStr">
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>CAMEL</t>
+        </is>
+      </c>
+      <c r="AK33" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="AM33" t="inlineStr">
         <is>
           <t>WOMEN</t>
         </is>
       </c>
-      <c r="AN31" t="inlineStr">
-        <is>
-          <t>712360626311804</t>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>184582324550</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>46092</v>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>46094</v>
+      </c>
+      <c r="D34" t="n">
+        <v>2000440</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Prepack SKU</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>JCPenney</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>JCPenney</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>JCPenney ( JC Penney (By CommerceHub) )</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>30007-260311-000013</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>ADELINE-02-CAMEL-A12</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>WOVEN SLIDE SANDAL</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>WOVEN SLIDE SANDAL</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>4</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" t="n">
+        <v>4</v>
+      </c>
+      <c r="U34" t="n">
+        <v>4</v>
+      </c>
+      <c r="V34" s="5" t="n">
+        <v>120.28</v>
+      </c>
+      <c r="W34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" s="5" t="n">
+        <v>120.28</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>ADELINE-02</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>CAMEL</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>WOMEN</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>582947026906</t>
         </is>
       </c>
     </row>

</xml_diff>